<commit_message>
Add EMEA/IL M365 group rows for all IL divisions/departments
For every HQ/IL row in All_365_Groups.xlsx that lacked a matching
EMEA/IL row, added the equivalent EMEA row (HQ_ prefix replaced
with EMEA_). Covers 28 new combinations so EMEA-region IL employees
are assigned the correct EMEA_* groups automatically.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/All_365_Groups.xlsx
+++ b/All_365_Groups.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J157"/>
+  <dimension ref="A1:J185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8596,6 +8596,1462 @@
         </is>
       </c>
     </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>IL_FIN_FIN@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>EMEA_FIN_FIN@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>EMEA_FIN@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>Global_FIN@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>Global_FIN_FIN@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>IL_OPS_IT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>EMEA_OPS_IT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>EMEA_OPS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>Global_OPS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>Global_OPS_IT@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>IL_PNT_RNDSW@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>EMEA_PNT_RNDSW@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>EMEA_PNT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>Global_PNT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>Global_PNT_RNDSW@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>V&amp;V &amp; QA</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>IL_PNT_VNVQA@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>EMEA_PNT_VNVQA@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>EMEA_PNT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>Global_PNT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>Global_PNT_VNVQA@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>IL_FIN_Admin@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>EMEA_FIN_Admin@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>EMEA_FIN@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>Global_FIN@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>Global_FIN_Admin@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Human Resources</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Human Resources</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>IL_HR_HR@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>EMEA_HR_HR@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>EMEA_HR@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>Global_HR@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>Global_HR_HR@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>IL_PNT_RNDHW@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>EMEA_PNT_RNDHW@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>EMEA_PNT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>Global_PNT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>Global_PNT_RNDHW@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>IL_OPS_ENG@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>EMEA_OPS_ENG@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>EMEA_OPS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>Global_OPS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>Global_OPS_ENG@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Management</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Management</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>IL_MGMT_MGMT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>EMEA_MGMT_MGMT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>EMEA_MGMT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>Global_MGMT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>Global_MGMT_MGMT@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Management</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>BD</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>IL_MGMT_BD@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>EMEA_MGMT_BD@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>EMEA_MGMT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>Global_MGMT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>Global_MGMT_BD@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Sales People</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>IL_MKT_SLS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>EMEA_MKT_SLS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>EMEA_MKT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>Global_MKT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>Global_MKT_SLS@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Products &amp; Solutions</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>IL_PNT_PNS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>EMEA_PNT_PNS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>EMEA_PNT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>Global_PNT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>Global_PNT_PNS@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Project Management</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>IL_PNT_PM@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>EMEA_PNT_PM@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>EMEA_PNT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>Global_PNT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>Global_PNT_PM@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Management</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>RND</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>IL_MGMT_RND@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>EMEA_MGMT_RND@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>EMEA_MGMT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>Global_MGMT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>Global_MGMT_RND@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>IL_MKT_MKT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>EMEA_MKT_MKT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>EMEA_MKT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>Global_MKT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>Global_MKT_MKT@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Purchasing</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>IL_OPS_PRC@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>EMEA_OPS_PRC@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>EMEA_OPS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>Global_OPS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>Global_OPS_PRC@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Management</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Human Resources</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>IL_MGMT_HR@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>EMEA_MGMT_HR@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>EMEA_MGMT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>Global_MGMT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>Global_MGMT_HR@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Planning</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>IL_OPS_PLN@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>EMEA_OPS_PLN@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>EMEA_OPS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>Global_OPS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>Global_OPS_PLN@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>IL_OPS_QA@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>EMEA_OPS_QA@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>EMEA_OPS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>Global_OPS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>Global_OPS_QA@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Management</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>IL_MGMT_Admin@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>EMEA_MGMT_Admin@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>EMEA_MGMT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>Global_MGMT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>Global_MGMT_Admin@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Management</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>IL_MGMT_MKT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>EMEA_MGMT_MKT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>EMEA_MGMT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>Global_MGMT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>Global_MGMT_MKT@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Management</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Products &amp; Solutions</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>IL_MGMT_PNS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>EMEA_MGMT_PNS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>EMEA_MGMT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>Global_MGMT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>Global_MGMT_PNS@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Products &amp; Solutions</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Products &amp; Solutions</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>IL_PNS_PNS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>EMEA_PNS_PNS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>EMEA_PNT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>Global_PNS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>Global_PNS_PNS@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Products &amp; Solutions</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Technical Writing</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>IL_PNS_PNS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>EMEA_PNS_PNS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>EMEA_PNT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>Global_PNS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>Global_PNS_PNS@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Customer Service</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>IL_PNT_CS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>EMEA_PNT_CS@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>EMEA_PNT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>Global_PNT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>Global_PNT_CS@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Management</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Product &amp; Technology</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>IL_MGMT_PNT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>EMEA_MGMT_PNT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>EMEA_MGMT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>Global_MGMT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>Global_MGMT_PNT@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Software - Embedded</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>IL_PNT_RNDSW@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>EMEA_PNT_RNDSW@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>EMEA_PNT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>Global_PNT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>Global_PNT_RNDSW@kramerav.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Software QA</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>IL_All_Employees@kramerav.com</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>IL_PNT_RNDSW@kramerav.com</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>EMEA_PNT_RNDSW@kramerav.com</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>EMEA_PNT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>Global_PNT@kramerav.com</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>Global_PNT_RNDSW@kramerav.com</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>